<commit_message>
updated after match 7
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65B4BB4-F8EC-4022-9401-6D18BB2BE06C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD4355E1-13A6-4CF4-86C0-9D036F586430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1057,61 +1057,61 @@
         <v>1</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>2</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1">
+        <v>29</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="1">
-        <v>0</v>
-      </c>
-      <c r="I3" s="1">
-        <v>48</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="M3" s="1">
-        <v>0</v>
-      </c>
-      <c r="N3" s="1">
-        <v>159</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="R3" s="1">
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>161</v>
+        <v>34</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>1</v>
@@ -1132,46 +1132,46 @@
         <v>1</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="AF3" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="AG3" s="1">
         <v>0</v>
       </c>
       <c r="AH3" s="1">
-        <v>162</v>
+        <v>25</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ3" s="1" t="s">
-        <v>117</v>
+        <v>45</v>
       </c>
       <c r="AK3" s="1" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="AL3" s="1">
         <v>0</v>
       </c>
       <c r="AM3" s="1">
-        <v>158</v>
+        <v>64</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="AQ3" s="1">
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
@@ -1191,76 +1191,76 @@
         <v>1</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H4" s="1">
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>143</v>
+        <v>14</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="L4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0</v>
+      </c>
+      <c r="N4" s="1">
+        <v>159</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0</v>
+      </c>
+      <c r="S4" s="1">
+        <v>54</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="M4" s="1">
-        <v>0</v>
-      </c>
-      <c r="N4" s="1">
-        <v>29</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="R4" s="1">
-        <v>0</v>
-      </c>
-      <c r="S4" s="1">
-        <v>34</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="W4" s="1">
         <v>0</v>
       </c>
       <c r="X4" s="1">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>81</v>
+        <v>52</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>1</v>
@@ -1281,31 +1281,31 @@
         <v>1</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="AK4" s="1" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="AL4" s="1">
         <v>0</v>
       </c>
       <c r="AM4" s="1">
-        <v>73</v>
+        <v>158</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>10</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
@@ -1325,31 +1325,31 @@
         <v>1</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>102</v>
+        <v>38</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>2</v>
+        <v>140</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
       </c>
       <c r="N5" s="1">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>1</v>
@@ -1370,31 +1370,31 @@
         <v>1</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>1</v>
@@ -1415,31 +1415,31 @@
         <v>1</v>
       </c>
       <c r="AJ5" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AK5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AL5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM5" s="1">
         <v>73</v>
       </c>
-      <c r="AK5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AL5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM5" s="1">
-        <v>211</v>
-      </c>
       <c r="AN5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1459,7 +1459,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>41</v>
@@ -1468,22 +1468,22 @@
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>54</v>
+        <v>145</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>1</v>
@@ -1504,10 +1504,10 @@
         <v>1</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="W6" s="1">
         <v>0</v>
@@ -1519,16 +1519,16 @@
         <v>1</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>115</v>
+        <v>32</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="AB6" s="1">
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>1</v>
@@ -1549,31 +1549,31 @@
         <v>1</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="AL6" s="1">
         <v>0</v>
       </c>
       <c r="AM6" s="1">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>0</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1593,25 +1593,25 @@
         <v>1</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>122</v>
+        <v>15</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>145</v>
+        <v>18</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="M7" s="1">
         <v>0</v>
@@ -1638,61 +1638,61 @@
         <v>1</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>17</v>
+        <v>167</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="AA7" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="AB7" s="1">
         <v>0</v>
       </c>
       <c r="AC7" s="1">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="AD7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>107</v>
+        <v>23</v>
       </c>
       <c r="AF7" s="1" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="AG7" s="1">
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>72</v>
+        <v>162</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="AK7" s="1" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="AL7" s="1">
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>1</v>
@@ -1721,37 +1721,37 @@
         <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="M8" s="1">
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>1</v>
@@ -1772,22 +1772,22 @@
         <v>1</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>106</v>
+        <v>52</v>
       </c>
       <c r="AA8" s="1" t="s">
         <v>25</v>
@@ -1802,46 +1802,46 @@
         <v>1</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="AG8" s="1">
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="AL8" s="1">
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>80</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
@@ -1861,16 +1861,16 @@
         <v>1</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>1</v>
@@ -1891,37 +1891,37 @@
         <v>1</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="R9" s="1">
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>12</v>
+        <v>161</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="W9" s="1">
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>152</v>
+        <v>108</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="AA9" s="1" t="s">
         <v>22</v>
@@ -1930,52 +1930,52 @@
         <v>0</v>
       </c>
       <c r="AC9" s="1">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="AD9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>130</v>
+        <v>44</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ9" s="1" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="AL9" s="1">
         <v>0</v>
       </c>
       <c r="AM9" s="1">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="AN9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="AP9" s="1" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="AQ9" s="1">
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -1995,10 +1995,10 @@
         <v>1</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H10" s="1">
         <v>0</v>
@@ -2010,40 +2010,40 @@
         <v>1</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="R10" s="1">
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="W10" s="1">
         <v>0</v>
@@ -2055,90 +2055,90 @@
         <v>1</v>
       </c>
       <c r="Z10" s="1" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="AA10" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="AB10" s="1">
         <v>0</v>
       </c>
       <c r="AC10" s="1">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="AG10" s="1">
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>58</v>
+        <v>114</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ10" s="1" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="AK10" s="1" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="AL10" s="1">
         <v>0</v>
       </c>
       <c r="AM10" s="1">
-        <v>0</v>
+        <v>211</v>
       </c>
       <c r="AN10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>46</v>
+        <v>121</v>
       </c>
       <c r="AP10" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="AQ10" s="1">
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>110</v>
+        <v>47</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1">
+        <v>118</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="1">
-        <v>0</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="H11" s="1">
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>1</v>
@@ -2174,120 +2174,120 @@
         <v>1</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="AA11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB11" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="1">
+        <v>81</v>
+      </c>
+      <c r="AD11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="AF11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AG11" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="1">
+        <v>130</v>
+      </c>
+      <c r="AI11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ11" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AK11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AL11" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM11" s="1">
+        <v>89</v>
+      </c>
+      <c r="AN11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AO11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AP11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AQ11" s="1">
+        <v>0</v>
+      </c>
+      <c r="AR11" s="1">
         <v>18</v>
-      </c>
-      <c r="AB11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC11" s="1">
-        <v>30</v>
-      </c>
-      <c r="AD11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AE11" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="AF11" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="1">
-        <v>114</v>
-      </c>
-      <c r="AI11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AK11" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM11" s="1">
-        <v>72</v>
-      </c>
-      <c r="AN11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AO11" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AP11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AQ11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AR11" s="1">
-        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>47</v>
+        <v>110</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F12" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
         <v>48</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H12" s="1">
-        <v>0</v>
-      </c>
-      <c r="I12" s="1">
-        <v>14</v>
-      </c>
       <c r="J12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>1</v>
@@ -2308,16 +2308,16 @@
         <v>1</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="W12" s="1">
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>8</v>
+        <v>120</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>1</v>
@@ -2332,52 +2332,52 @@
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>2</v>
+        <v>145</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AE12" s="1" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="AF12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH12" s="1">
+        <v>58</v>
+      </c>
+      <c r="AI12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AL12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM12" s="1">
+        <v>98</v>
+      </c>
+      <c r="AN12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AO12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AP12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AG12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="1">
-        <v>2</v>
-      </c>
-      <c r="AI12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ12" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="AK12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="AL12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AN12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AO12" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="AP12" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="AQ12" s="1">
         <v>0</v>
       </c>
       <c r="AR12" s="1">
-        <v>18</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2397,16 +2397,16 @@
         <v>1</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H13" s="1">
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>86</v>
+        <v>143</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>1</v>
@@ -2436,37 +2436,37 @@
         <v>0</v>
       </c>
       <c r="S13" s="1">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="W13" s="1">
         <v>0</v>
       </c>
       <c r="X13" s="1">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z13" s="1" t="s">
-        <v>71</v>
+        <v>115</v>
       </c>
       <c r="AA13" s="1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="AB13" s="1">
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>19</v>
+        <v>127</v>
       </c>
       <c r="AD13" s="1" t="s">
         <v>1</v>
@@ -2487,16 +2487,16 @@
         <v>1</v>
       </c>
       <c r="AJ13" s="1" t="s">
-        <v>123</v>
+        <v>54</v>
       </c>
       <c r="AK13" s="1" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="AL13" s="1">
         <v>0</v>
       </c>
       <c r="AM13" s="1">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="AN13" s="1" t="s">
         <v>1</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>1</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>535</v>
+        <v>589</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>466</v>
+        <v>531</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>1</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>354</v>
+        <v>390</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>1</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>767</v>
+        <v>912</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>1</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>446</v>
+        <v>795</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>1</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>659</v>
+        <v>682</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>1</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>781</v>
+        <v>795</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>1</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>481</v>
+        <v>653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 8
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD4355E1-13A6-4CF4-86C0-9D036F586430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A9EBFC-D456-4EE2-8D50-9C1FB57B558D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1087,61 +1087,61 @@
         <v>1</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="R3" s="1">
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>62</v>
+        <v>164</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB3" s="1">
         <v>0</v>
       </c>
       <c r="AC3" s="1">
-        <v>28</v>
+        <v>96</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="AF3" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="AG3" s="1">
         <v>0</v>
       </c>
       <c r="AH3" s="1">
-        <v>25</v>
+        <v>233</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>1</v>
@@ -1156,22 +1156,22 @@
         <v>0</v>
       </c>
       <c r="AM3" s="1">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AQ3" s="1">
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>80</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
@@ -1191,16 +1191,16 @@
         <v>1</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="H4" s="1">
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>14</v>
+        <v>140</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>1</v>
@@ -1221,46 +1221,46 @@
         <v>1</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="Q4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0</v>
+      </c>
+      <c r="S4" s="1">
+        <v>25</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="W4" s="1">
+        <v>0</v>
+      </c>
+      <c r="X4" s="1">
+        <v>108</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="R4" s="1">
-        <v>0</v>
-      </c>
-      <c r="S4" s="1">
-        <v>54</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="W4" s="1">
-        <v>0</v>
-      </c>
-      <c r="X4" s="1">
-        <v>72</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>1</v>
@@ -1275,37 +1275,37 @@
         <v>0</v>
       </c>
       <c r="AH4" s="1">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>117</v>
+        <v>64</v>
       </c>
       <c r="AK4" s="1" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="AL4" s="1">
         <v>0</v>
       </c>
       <c r="AM4" s="1">
-        <v>158</v>
+        <v>108</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
@@ -1325,67 +1325,67 @@
         <v>1</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>140</v>
+        <v>9</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
       </c>
       <c r="N5" s="1">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="R5" s="1">
         <v>0</v>
       </c>
       <c r="S5" s="1">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>20</v>
+        <v>114</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="AA5" s="1" t="s">
         <v>22</v>
@@ -1394,7 +1394,7 @@
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>1</v>
@@ -1415,31 +1415,31 @@
         <v>1</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>108</v>
+        <v>34</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1459,40 +1459,40 @@
         <v>1</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>122</v>
+        <v>15</v>
       </c>
       <c r="G6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>18</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0</v>
+      </c>
+      <c r="N6" s="1">
+        <v>0</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q6" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="H6" s="1">
-        <v>0</v>
-      </c>
-      <c r="I6" s="1">
-        <v>145</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="M6" s="1">
-        <v>0</v>
-      </c>
-      <c r="N6" s="1">
-        <v>33</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="R6" s="1">
         <v>0</v>
@@ -1519,7 +1519,7 @@
         <v>1</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="AA6" s="1" t="s">
         <v>22</v>
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>1</v>
@@ -1564,16 +1564,16 @@
         <v>1</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1593,91 +1593,91 @@
         <v>1</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>15</v>
+        <v>122</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
+        <v>145</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M7" s="1">
-        <v>0</v>
-      </c>
-      <c r="N7" s="1">
-        <v>0</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q7" s="1" t="s">
+      <c r="R7" s="1">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1">
+        <v>0</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="V7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="R7" s="1">
-        <v>0</v>
-      </c>
-      <c r="S7" s="1">
-        <v>0</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="W7" s="1">
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>167</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="AA7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AB7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="1">
-        <v>19</v>
-      </c>
-      <c r="AD7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AE7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AF7" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="AG7" s="1">
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>1</v>
@@ -1698,105 +1698,105 @@
         <v>1</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="AP7" s="1" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="AQ7" s="1">
         <v>0</v>
       </c>
       <c r="AR7" s="1">
-        <v>0</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
       </c>
       <c r="D8" s="1">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
+        <v>25</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8" s="1">
+        <v>0</v>
+      </c>
+      <c r="N8" s="1">
+        <v>98</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R8" s="1">
+        <v>0</v>
+      </c>
+      <c r="S8" s="1">
+        <v>0</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" s="1">
-        <v>0</v>
-      </c>
-      <c r="I8" s="1">
-        <v>54</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M8" s="1">
-        <v>0</v>
-      </c>
-      <c r="N8" s="1">
-        <v>0</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="R8" s="1">
-        <v>0</v>
-      </c>
-      <c r="S8" s="1">
-        <v>10</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AB8" s="1">
         <v>0</v>
       </c>
       <c r="AC8" s="1">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>1</v>
@@ -1817,16 +1817,16 @@
         <v>1</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>34</v>
+        <v>117</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="AL8" s="1">
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>72</v>
+        <v>158</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>1</v>
@@ -1846,159 +1846,159 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0</v>
+      </c>
+      <c r="N9" s="1">
+        <v>34</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="R9" s="1">
+        <v>0</v>
+      </c>
+      <c r="S9" s="1">
+        <v>10</v>
+      </c>
+      <c r="T9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="V9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="W9" s="1">
+        <v>0</v>
+      </c>
+      <c r="X9" s="1">
+        <v>194</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="1">
+        <v>19</v>
+      </c>
+      <c r="AD9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AF9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AG9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="1">
         <v>25</v>
       </c>
-      <c r="C9" s="1">
-        <v>0</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="1">
-        <v>0</v>
-      </c>
-      <c r="I9" s="1">
-        <v>25</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M9" s="1">
-        <v>0</v>
-      </c>
-      <c r="N9" s="1">
-        <v>98</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="R9" s="1">
-        <v>0</v>
-      </c>
-      <c r="S9" s="1">
-        <v>161</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="W9" s="1">
-        <v>0</v>
-      </c>
-      <c r="X9" s="1">
+      <c r="AI9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ9" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="Y9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="Z9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AB9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="1">
-        <v>56</v>
-      </c>
-      <c r="AD9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AE9" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AF9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AG9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH9" s="1">
-        <v>44</v>
-      </c>
-      <c r="AI9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ9" s="1" t="s">
+      <c r="AK9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AL9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="1">
+        <v>73</v>
+      </c>
+      <c r="AN9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AO9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AP9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AQ9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AR9" s="1">
         <v>99</v>
-      </c>
-      <c r="AK9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="AL9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM9" s="1">
-        <v>14</v>
-      </c>
-      <c r="AN9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AO9" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="AP9" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AQ9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AR9" s="1">
-        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="H10" s="1">
         <v>0</v>
@@ -2025,16 +2025,16 @@
         <v>1</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="R10" s="1">
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>12</v>
+        <v>161</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>1</v>
@@ -2100,45 +2100,45 @@
         <v>1</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>121</v>
+        <v>74</v>
       </c>
       <c r="AP10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AQ10" s="1">
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>47</v>
+        <v>110</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>1</v>
@@ -2159,46 +2159,46 @@
         <v>1</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="R11" s="1">
         <v>0</v>
       </c>
       <c r="S11" s="1">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>152</v>
+        <v>57</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
       </c>
       <c r="AC11" s="1">
-        <v>81</v>
+        <v>52</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>1</v>
@@ -2213,51 +2213,51 @@
         <v>0</v>
       </c>
       <c r="AH11" s="1">
-        <v>130</v>
+        <v>188</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ11" s="1" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="AK11" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="AL11" s="1">
         <v>0</v>
       </c>
       <c r="AM11" s="1">
-        <v>89</v>
+        <v>14</v>
       </c>
       <c r="AN11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>74</v>
+        <v>118</v>
       </c>
       <c r="AP11" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="AQ11" s="1">
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>110</v>
+        <v>47</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>1</v>
@@ -2278,61 +2278,61 @@
         <v>1</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="L12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="N12" s="1">
+        <v>78</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="R12" s="1">
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
+        <v>43</v>
+      </c>
+      <c r="T12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="V12" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="1">
-        <v>0</v>
-      </c>
-      <c r="N12" s="1">
-        <v>69</v>
-      </c>
-      <c r="O12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R12" s="1">
-        <v>0</v>
-      </c>
-      <c r="S12" s="1">
-        <v>12</v>
-      </c>
-      <c r="T12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U12" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="W12" s="1">
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="AB12" s="1">
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>1</v>
@@ -2347,22 +2347,22 @@
         <v>0</v>
       </c>
       <c r="AH12" s="1">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="AI12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>64</v>
+        <v>123</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AL12" s="1">
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>1</v>
@@ -2382,16 +2382,16 @@
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C13" s="1">
         <v>0</v>
       </c>
       <c r="D13" s="1">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>1</v>
@@ -2412,61 +2412,61 @@
         <v>1</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>28</v>
+        <v>94</v>
       </c>
       <c r="L13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="N13" s="1">
+        <v>69</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="1">
-        <v>0</v>
-      </c>
-      <c r="N13" s="1">
-        <v>78</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q13" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="R13" s="1">
         <v>0</v>
       </c>
       <c r="S13" s="1">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="W13" s="1">
         <v>0</v>
       </c>
       <c r="X13" s="1">
-        <v>63</v>
+        <v>152</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z13" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AA13" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AB13" s="1">
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="AD13" s="1" t="s">
         <v>1</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>434</v>
+        <v>475</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>1</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>1</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>390</v>
+        <v>454</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>1</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>912</v>
+        <v>978</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>1</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>795</v>
+        <v>810</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>1</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>682</v>
+        <v>910</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>1</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>795</v>
+        <v>869</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>1</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>653</v>
+        <v>658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 14
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8805665B-69BC-44A8-B96E-C02CF1CCD869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E41C96-3740-4929-923E-17CC02A2D6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="AM3" s="1">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>123</v>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>123</v>
@@ -1439,7 +1439,7 @@
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>78</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1534,16 +1534,16 @@
         <v>123</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="AF6" s="1" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="AG6" s="1">
         <v>0</v>
       </c>
       <c r="AH6" s="1">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="AI6" s="1" t="s">
         <v>123</v>
@@ -1573,7 +1573,7 @@
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>92</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1668,10 +1668,10 @@
         <v>123</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>88</v>
+        <v>52</v>
       </c>
       <c r="AF7" s="1" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="AG7" s="1">
         <v>0</v>
@@ -1802,16 +1802,16 @@
         <v>123</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="AG8" s="1">
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>294</v>
+        <v>0</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>123</v>
@@ -1936,16 +1936,16 @@
         <v>123</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>177</v>
+        <v>294</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
@@ -2064,22 +2064,22 @@
         <v>0</v>
       </c>
       <c r="AC10" s="1">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AG10" s="1">
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>123</v>
@@ -2094,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="AM10" s="1">
-        <v>89</v>
+        <v>229</v>
       </c>
       <c r="AN10" s="1" t="s">
         <v>123</v>
@@ -2204,16 +2204,16 @@
         <v>123</v>
       </c>
       <c r="AE11" s="1" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="AF11" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="AG11" s="1">
         <v>0</v>
       </c>
       <c r="AH11" s="1">
-        <v>213</v>
+        <v>248</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>123</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>53</v>
+        <v>140</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>123</v>
@@ -2302,7 +2302,7 @@
         <v>0</v>
       </c>
       <c r="S12" s="1">
-        <v>144</v>
+        <v>282</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>123</v>
@@ -2317,7 +2317,7 @@
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>123</v>
@@ -2332,22 +2332,22 @@
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE12" s="1" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="AF12" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="AG12" s="1">
         <v>0</v>
       </c>
       <c r="AH12" s="1">
-        <v>25</v>
+        <v>213</v>
       </c>
       <c r="AI12" s="1" t="s">
         <v>123</v>
@@ -2377,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="AR12" s="1">
-        <v>15</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2421,7 +2421,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="1">
-        <v>146</v>
+        <v>278</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>123</v>
@@ -2472,16 +2472,16 @@
         <v>123</v>
       </c>
       <c r="AE13" s="1" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AF13" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AG13" s="1">
         <v>0</v>
       </c>
       <c r="AH13" s="1">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="AI13" s="1" t="s">
         <v>123</v>
@@ -2496,7 +2496,7 @@
         <v>0</v>
       </c>
       <c r="AM13" s="1">
-        <v>108</v>
+        <v>159</v>
       </c>
       <c r="AN13" s="1" t="s">
         <v>123</v>
@@ -2511,7 +2511,7 @@
         <v>0</v>
       </c>
       <c r="AR13" s="1">
-        <v>184</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>662</v>
+        <v>749</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>123</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>1100</v>
+        <v>1142</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>123</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>935</v>
+        <v>1067</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>123</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>972</v>
+        <v>1110</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>123</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>1216</v>
+        <v>1228</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>123</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>980</v>
+        <v>1004</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>123</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>1456</v>
+        <v>1576</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>123</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>1527</v>
+        <v>1726</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>123</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>1160</v>
+        <v>1569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 15
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E41C96-3740-4929-923E-17CC02A2D6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0700913F-D003-4958-839D-60F94282E261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>167</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
@@ -1185,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>52</v>
+        <v>144</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>123</v>
@@ -1245,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="X4" s="1">
-        <v>84</v>
+        <v>154</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>123</v>
@@ -1647,7 +1647,7 @@
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>123</v>
@@ -1751,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>123</v>
@@ -1781,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>123</v>
@@ -1826,7 +1826,7 @@
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>123</v>
@@ -1885,7 +1885,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>22</v>
+        <v>132</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>123</v>
@@ -1975,7 +1975,7 @@
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>86</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -2034,7 +2034,7 @@
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>123</v>
@@ -2228,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="AM11" s="1">
-        <v>211</v>
+        <v>306</v>
       </c>
       <c r="AN11" s="1" t="s">
         <v>123</v>
@@ -2287,7 +2287,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>123</v>
@@ -2362,7 +2362,7 @@
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>123</v>
@@ -2406,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>143</v>
+        <v>226</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>123</v>
@@ -2451,7 +2451,7 @@
         <v>0</v>
       </c>
       <c r="X13" s="1">
-        <v>171</v>
+        <v>206</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>123</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>749</v>
+        <v>841</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>123</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>1142</v>
+        <v>1225</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>123</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>1067</v>
+        <v>1258</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>123</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>1110</v>
+        <v>1131</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>123</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>1228</v>
+        <v>1355</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>123</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>1726</v>
+        <v>1906</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>123</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>1569</v>
+        <v>1648</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 21
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EEC387-F32A-4301-9CBB-795D9BF9831C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B58F36-5983-4030-B1BD-0155BA6664B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1061,7 +1061,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="E3" t="s">
         <v>123</v>
@@ -1106,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <v>402</v>
+        <v>417</v>
       </c>
       <c r="T3" t="s">
         <v>123</v>
@@ -1142,16 +1142,16 @@
         <v>123</v>
       </c>
       <c r="AE3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="AF3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AG3">
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>281</v>
+        <v>124</v>
       </c>
       <c r="AI3" t="s">
         <v>123</v>
@@ -1225,7 +1225,7 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <v>334</v>
+        <v>408</v>
       </c>
       <c r="O4" t="s">
         <v>123</v>
@@ -1240,7 +1240,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="T4" t="s">
         <v>123</v>
@@ -1276,7 +1276,7 @@
         <v>123</v>
       </c>
       <c r="AE4" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="AF4" t="s">
         <v>15</v>
@@ -1285,7 +1285,7 @@
         <v>0</v>
       </c>
       <c r="AH4">
-        <v>125</v>
+        <v>281</v>
       </c>
       <c r="AI4" t="s">
         <v>123</v>
@@ -1410,7 +1410,7 @@
         <v>123</v>
       </c>
       <c r="AE5" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="AF5" t="s">
         <v>15</v>
@@ -1419,7 +1419,7 @@
         <v>0</v>
       </c>
       <c r="AH5">
-        <v>208</v>
+        <v>125</v>
       </c>
       <c r="AI5" t="s">
         <v>123</v>
@@ -1538,13 +1538,13 @@
         <v>0</v>
       </c>
       <c r="AC6">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="AD6" t="s">
         <v>123</v>
       </c>
       <c r="AE6" t="s">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="AF6" t="s">
         <v>23</v>
@@ -1553,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="AH6">
-        <v>124</v>
+        <v>243</v>
       </c>
       <c r="AI6" t="s">
         <v>123</v>
@@ -1678,16 +1678,16 @@
         <v>123</v>
       </c>
       <c r="AE7" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="AF7" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="AG7">
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="AI7" t="s">
         <v>123</v>
@@ -1717,7 +1717,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
@@ -1761,7 +1761,7 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>194</v>
+        <v>269</v>
       </c>
       <c r="O8" t="s">
         <v>123</v>
@@ -1812,10 +1812,10 @@
         <v>123</v>
       </c>
       <c r="AE8" t="s">
-        <v>88</v>
+        <v>52</v>
       </c>
       <c r="AF8" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="AG8">
         <v>0</v>
@@ -1836,7 +1836,7 @@
         <v>0</v>
       </c>
       <c r="AM8">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="AN8" t="s">
         <v>123</v>
@@ -1946,16 +1946,16 @@
         <v>123</v>
       </c>
       <c r="AE9" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="AF9" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AG9">
         <v>0</v>
       </c>
       <c r="AH9">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="AI9" t="s">
         <v>123</v>
@@ -1985,7 +1985,7 @@
         <v>0</v>
       </c>
       <c r="AR9">
-        <v>289</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -2080,16 +2080,16 @@
         <v>123</v>
       </c>
       <c r="AE10" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="AF10" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="AG10">
         <v>0</v>
       </c>
       <c r="AH10">
-        <v>384</v>
+        <v>265</v>
       </c>
       <c r="AI10" t="s">
         <v>123</v>
@@ -2104,7 +2104,7 @@
         <v>0</v>
       </c>
       <c r="AM10">
-        <v>294</v>
+        <v>384</v>
       </c>
       <c r="AN10" t="s">
         <v>123</v>
@@ -2214,16 +2214,16 @@
         <v>123</v>
       </c>
       <c r="AE11" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="AF11" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AG11">
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>243</v>
+        <v>384</v>
       </c>
       <c r="AI11" t="s">
         <v>123</v>
@@ -2253,7 +2253,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
@@ -2267,7 +2267,7 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <v>296</v>
+        <v>475</v>
       </c>
       <c r="E12" t="s">
         <v>123</v>
@@ -2282,7 +2282,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="J12" t="s">
         <v>123</v>
@@ -2357,7 +2357,7 @@
         <v>0</v>
       </c>
       <c r="AH12">
-        <v>287</v>
+        <v>375</v>
       </c>
       <c r="AI12" t="s">
         <v>123</v>
@@ -2461,7 +2461,7 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>264</v>
+        <v>286</v>
       </c>
       <c r="Y13" t="s">
         <v>123</v>
@@ -2476,7 +2476,7 @@
         <v>0</v>
       </c>
       <c r="AC13">
-        <v>218</v>
+        <v>250</v>
       </c>
       <c r="AD13" t="s">
         <v>123</v>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="D14">
         <f>SUM(D3:D13)</f>
-        <v>1150</v>
+        <v>1331</v>
       </c>
       <c r="E14" t="s">
         <v>123</v>
@@ -2551,8 +2551,7 @@
         <v>0</v>
       </c>
       <c r="I14">
-        <f>SUM(I3:I13)</f>
-        <v>1792</v>
+        <v>1800</v>
       </c>
       <c r="J14" t="s">
         <v>123</v>
@@ -2568,7 +2567,7 @@
       </c>
       <c r="N14">
         <f>SUM(N3:N13)</f>
-        <v>2018</v>
+        <v>2167</v>
       </c>
       <c r="O14" t="s">
         <v>123</v>
@@ -2584,7 +2583,7 @@
       </c>
       <c r="S14">
         <f>SUM(S3:S13)</f>
-        <v>1765</v>
+        <v>1778</v>
       </c>
       <c r="T14" t="s">
         <v>123</v>
@@ -2599,8 +2598,7 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <f>SUM(X3:X13)</f>
-        <v>1809</v>
+        <v>1831</v>
       </c>
       <c r="Y14" t="s">
         <v>123</v>
@@ -2616,7 +2614,7 @@
       </c>
       <c r="AC14">
         <f>SUM(AC3:AC13)</f>
-        <v>1633</v>
+        <v>1685</v>
       </c>
       <c r="AD14" t="s">
         <v>123</v>
@@ -2632,7 +2630,7 @@
       </c>
       <c r="AH14">
         <f>SUM(AH3:AH13)</f>
-        <v>1951</v>
+        <v>2039</v>
       </c>
       <c r="AI14" t="s">
         <v>123</v>
@@ -2648,7 +2646,7 @@
       </c>
       <c r="AM14">
         <f>SUM(AM3:AM13)</f>
-        <v>2441</v>
+        <v>2536</v>
       </c>
       <c r="AN14" t="s">
         <v>123</v>
@@ -2664,7 +2662,7 @@
       </c>
       <c r="AR14">
         <f>SUM(AR3:AR13)</f>
-        <v>2512</v>
+        <v>2514</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 23
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BEB1AE-5696-45C3-91A3-BDE3741DFA07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50892927-91B2-432B-845E-0DE70E476D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3348" yWindow="3348" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1098,31 +1098,31 @@
         <v>123</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="R3" s="1">
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>417</v>
+        <v>119</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>123</v>
@@ -1182,7 +1182,7 @@
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
@@ -1202,16 +1202,16 @@
         <v>123</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>47</v>
+        <v>121</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H4" s="1">
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>103</v>
+        <v>470</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>123</v>
@@ -1232,31 +1232,31 @@
         <v>123</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>95</v>
+        <v>417</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>30</v>
+        <v>104</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="W4" s="1">
         <v>0</v>
       </c>
       <c r="X4" s="1">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>123</v>
@@ -1292,60 +1292,60 @@
         <v>123</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="AK4" s="1" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="AL4" s="1">
         <v>0</v>
       </c>
       <c r="AM4" s="1">
-        <v>165</v>
+        <v>512</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>0</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
       </c>
       <c r="D5" s="1">
-        <v>171</v>
+        <v>40</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>241</v>
+        <v>103</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>123</v>
@@ -1366,31 +1366,31 @@
         <v>123</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="Q5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R5" s="1">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
+        <v>95</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="R5" s="1">
-        <v>0</v>
-      </c>
-      <c r="S5" s="1">
-        <v>119</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>181</v>
+        <v>118</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>123</v>
@@ -1426,60 +1426,60 @@
         <v>123</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>256</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>40</v>
+        <v>171</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>61</v>
+        <v>241</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>123</v>
@@ -1500,31 +1500,31 @@
         <v>123</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="R6" s="1">
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>86</v>
+        <v>235</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="W6" s="1">
         <v>0</v>
       </c>
       <c r="X6" s="1">
-        <v>270</v>
+        <v>181</v>
       </c>
       <c r="Y6" s="1" t="s">
         <v>123</v>
@@ -1560,31 +1560,31 @@
         <v>123</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="AL6" s="1">
         <v>0</v>
       </c>
       <c r="AM6" s="1">
-        <v>439</v>
+        <v>0</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>239</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1604,16 +1604,16 @@
         <v>123</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>123</v>
@@ -1634,31 +1634,31 @@
         <v>123</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="R7" s="1">
         <v>0</v>
       </c>
       <c r="S7" s="1">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="T7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>38</v>
+        <v>270</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>123</v>
@@ -1694,31 +1694,31 @@
         <v>123</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="AK7" s="1" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="AL7" s="1">
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="AP7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AQ7" s="1">
         <v>0</v>
       </c>
       <c r="AR7" s="1">
-        <v>186</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
@@ -1738,16 +1738,16 @@
         <v>123</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>123</v>
@@ -1768,31 +1768,31 @@
         <v>123</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="R8" s="1">
         <v>0</v>
       </c>
       <c r="S8" s="1">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>235</v>
+        <v>38</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>123</v>
@@ -1828,22 +1828,22 @@
         <v>123</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="AL8" s="1">
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>392</v>
+        <v>97</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="AP8" s="1" t="s">
         <v>23</v>
@@ -1852,7 +1852,7 @@
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>254</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
@@ -1872,16 +1872,16 @@
         <v>123</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>121</v>
+        <v>37</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>381</v>
+        <v>148</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>123</v>
@@ -1896,13 +1896,13 @@
         <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>258</v>
+        <v>280</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>112</v>
+        <v>39</v>
       </c>
       <c r="Q9" s="1" t="s">
         <v>40</v>
@@ -1911,22 +1911,22 @@
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>69</v>
+        <v>160</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>113</v>
+        <v>50</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="W9" s="1">
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>136</v>
+        <v>235</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>123</v>
@@ -1962,31 +1962,31 @@
         <v>123</v>
       </c>
       <c r="AJ9" s="1" t="s">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="AL9" s="1">
         <v>0</v>
       </c>
       <c r="AM9" s="1">
-        <v>152</v>
+        <v>392</v>
       </c>
       <c r="AN9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="AP9" s="1" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AQ9" s="1">
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>299</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -2030,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>147</v>
+        <v>219</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>123</v>
@@ -2051,16 +2051,16 @@
         <v>123</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="W10" s="1">
         <v>0</v>
       </c>
       <c r="X10" s="1">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>123</v>
@@ -2096,31 +2096,31 @@
         <v>123</v>
       </c>
       <c r="AJ10" s="1" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="AK10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM10" s="1">
+        <v>166</v>
+      </c>
+      <c r="AN10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO10" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AP10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="AL10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM10" s="1">
-        <v>384</v>
-      </c>
-      <c r="AN10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO10" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="AP10" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="AQ10" s="1">
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>169</v>
+        <v>299</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
@@ -2149,7 +2149,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>235</v>
+        <v>365</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>123</v>
@@ -2179,22 +2179,22 @@
         <v>0</v>
       </c>
       <c r="S11" s="1">
-        <v>287</v>
+        <v>323</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>247</v>
+        <v>172</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>123</v>
@@ -2230,16 +2230,16 @@
         <v>123</v>
       </c>
       <c r="AJ11" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="AK11" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="AL11" s="1">
         <v>0</v>
       </c>
       <c r="AM11" s="1">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="AN11" s="1" t="s">
         <v>123</v>
@@ -2254,7 +2254,7 @@
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>211</v>
+        <v>303</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
@@ -2283,7 +2283,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>302</v>
+        <v>325</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>123</v>
@@ -2298,7 +2298,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>151</v>
+        <v>223</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>123</v>
@@ -2319,7 +2319,7 @@
         <v>123</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="V12" s="1" t="s">
         <v>15</v>
@@ -2328,7 +2328,7 @@
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>291</v>
+        <v>247</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>123</v>
@@ -2364,16 +2364,16 @@
         <v>123</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>72</v>
+        <v>122</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="AL12" s="1">
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>361</v>
+        <v>345</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>123</v>
@@ -2453,16 +2453,16 @@
         <v>123</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="W13" s="1">
         <v>0</v>
       </c>
       <c r="X13" s="1">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>123</v>
@@ -2498,16 +2498,16 @@
         <v>123</v>
       </c>
       <c r="AJ13" s="1" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="AK13" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="AL13" s="1">
         <v>0</v>
       </c>
       <c r="AM13" s="1">
-        <v>75</v>
+        <v>361</v>
       </c>
       <c r="AN13" s="1" t="s">
         <v>123</v>
@@ -2551,7 +2551,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>1848</v>
+        <v>2090</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>123</v>
@@ -2566,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>2391</v>
+        <v>2557</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>123</v>
@@ -2581,7 +2581,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>1870</v>
+        <v>2043</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>123</v>
@@ -2596,7 +2596,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>1974</v>
+        <v>1990</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>123</v>
@@ -2641,7 +2641,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>2591</v>
+        <v>2691</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>123</v>
@@ -2656,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>2551</v>
+        <v>2739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>